<commit_message>
feat: actualizar plantilla de excel chancado
</commit_message>
<xml_diff>
--- a/chancado/analytica/Report/Lote-Export-Base.xlsx
+++ b/chancado/analytica/Report/Lote-Export-Base.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\projects\minersoft-projects\minersoft\acopio-chancado-api\Acopio.Chancado.Apis\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0A63E41-8FB6-4A92-8979-920142A447F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7AE4F18-A650-4594-B271-F045A1860F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28908" yWindow="-108" windowWidth="29016" windowHeight="15696" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -161,7 +161,7 @@
     <numFmt numFmtId="165" formatCode="_-&quot;S/ &quot;* #,##0.00_-;&quot;-S/ &quot;* #,##0.00_-;_-&quot;S/ &quot;* \-??_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -281,6 +281,13 @@
     <font>
       <sz val="8"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -311,24 +318,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <fgColor theme="1"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor rgb="FF969696"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -355,33 +362,7 @@
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
       <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -418,7 +399,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="22" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -479,78 +460,74 @@
     <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="17" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="24" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="24" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="6" borderId="0" xfId="24" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="22" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="7" borderId="0" xfId="24" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="7" borderId="0" xfId="24" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="16" fontId="17" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="22" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="22" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="22" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="25">
@@ -580,93 +557,7 @@
     <cellStyle name="Normal 2 2 2 2" xfId="24" xr:uid="{7D02EEDF-F966-42E2-BF75-AE97ED01237A}"/>
     <cellStyle name="Normal 3" xfId="23" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
   </cellStyles>
-  <dxfs count="21">
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <numFmt numFmtId="21" formatCode="dd\-mmm"/>
-      <fill>
-        <gradientFill type="path" left="0.5" right="0.5" top="0.5" bottom="0.5">
-          <stop position="0">
-            <color rgb="FF00FF00"/>
-          </stop>
-          <stop position="1">
-            <color rgb="FF00B050"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFC0C0C0"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color theme="1"/>
-        </left>
-        <right style="thin">
-          <color theme="1"/>
-        </right>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom style="thin">
-          <color theme="1"/>
-        </bottom>
-      </border>
-    </dxf>
+  <dxfs count="10">
     <dxf>
       <font>
         <b/>
@@ -709,88 +600,12 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFC0C0C0"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color theme="1"/>
-        </left>
-        <right style="thin">
-          <color theme="1"/>
-        </right>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom style="thin">
-          <color theme="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <numFmt numFmtId="21" formatCode="dd\-mmm"/>
-      <fill>
-        <gradientFill type="path" left="0.5" right="0.5" top="0.5" bottom="0.5">
-          <stop position="0">
-            <color rgb="FF00FF00"/>
-          </stop>
-          <stop position="1">
-            <color rgb="FF00B050"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
+        <color auto="1"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFCC"/>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -815,14 +630,44 @@
         <color rgb="FFFF0000"/>
       </font>
       <fill>
-        <gradientFill degree="90">
-          <stop position="0">
-            <color theme="1"/>
-          </stop>
-          <stop position="1">
-            <color theme="0"/>
-          </stop>
-        </gradientFill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="1"/>
+        </left>
+        <right style="thin">
+          <color theme="1"/>
+        </right>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom style="thin">
+          <color theme="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF5D5D"/>
+        </patternFill>
       </fill>
     </dxf>
   </dxfs>
@@ -895,6 +740,7 @@
       <rgbColor rgb="00333333"/>
     </indexedColors>
     <mruColors>
+      <color rgb="FFFF5D5D"/>
       <color rgb="FF00FF00"/>
       <color rgb="FFC0C0C0"/>
       <color rgb="FFFFFFFF"/>
@@ -1090,38 +936,37 @@
   <dimension ref="A1:BF12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.77734375" style="23" customWidth="1"/>
-    <col min="2" max="2" width="19.77734375" style="24" customWidth="1"/>
-    <col min="3" max="3" width="19.5546875" style="25" customWidth="1"/>
-    <col min="4" max="4" width="19.5546875" style="23" customWidth="1"/>
-    <col min="5" max="5" width="16.6640625" style="23" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.77734375" style="23" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.5546875" style="26" customWidth="1"/>
-    <col min="8" max="8" width="10" style="26" customWidth="1"/>
-    <col min="9" max="9" width="9.109375" style="23" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="44.88671875" style="23" customWidth="1"/>
-    <col min="11" max="11" width="25.77734375" style="23" customWidth="1"/>
-    <col min="12" max="12" width="52.5546875" style="23" customWidth="1"/>
-    <col min="13" max="13" width="19.88671875" style="23" customWidth="1"/>
-    <col min="14" max="14" width="15" style="23" customWidth="1"/>
-    <col min="15" max="15" width="17.33203125" style="23" customWidth="1"/>
-    <col min="16" max="16" width="10.33203125" style="27" customWidth="1"/>
-    <col min="17" max="17" width="12.21875" style="27" customWidth="1"/>
-    <col min="18" max="18" width="10.44140625" style="24" customWidth="1"/>
-    <col min="19" max="19" width="12.5546875" style="24" customWidth="1"/>
-    <col min="20" max="20" width="10.6640625" style="28"/>
-    <col min="21" max="21" width="10.6640625" style="30"/>
-    <col min="22" max="22" width="10.6640625" style="31"/>
-    <col min="23" max="23" width="14.6640625" style="23" customWidth="1"/>
-    <col min="24" max="24" width="13.77734375" style="23" customWidth="1"/>
-    <col min="25" max="26" width="10.6640625" style="23"/>
-    <col min="27" max="27" width="22.109375" style="23" customWidth="1"/>
-    <col min="28" max="28" width="24.5546875" style="23" customWidth="1"/>
-    <col min="29" max="29" width="20.5546875" style="23" customWidth="1"/>
-    <col min="30" max="30" width="14.109375" style="32" customWidth="1"/>
-    <col min="31" max="31" width="18.5546875" style="23" customWidth="1"/>
-    <col min="32" max="32" width="27.109375" style="23" customWidth="1"/>
-    <col min="33" max="16384" width="10.6640625" style="22"/>
+    <col min="1" max="1" width="6.77734375" style="22" customWidth="1"/>
+    <col min="2" max="2" width="19.77734375" style="23" customWidth="1"/>
+    <col min="3" max="3" width="19.5546875" style="24" customWidth="1"/>
+    <col min="4" max="4" width="19.5546875" style="33" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" style="33" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.77734375" style="33" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.5546875" style="22" customWidth="1"/>
+    <col min="8" max="8" width="10" style="22" customWidth="1"/>
+    <col min="9" max="9" width="9.109375" style="33" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="44.88671875" style="33" customWidth="1"/>
+    <col min="11" max="11" width="25.77734375" style="33" customWidth="1"/>
+    <col min="12" max="12" width="52.5546875" style="33" customWidth="1"/>
+    <col min="13" max="13" width="19.88671875" style="33" customWidth="1"/>
+    <col min="14" max="14" width="15" style="33" customWidth="1"/>
+    <col min="15" max="15" width="17.33203125" style="33" customWidth="1"/>
+    <col min="16" max="16" width="10.33203125" style="25" customWidth="1"/>
+    <col min="17" max="17" width="12.21875" style="25" customWidth="1"/>
+    <col min="18" max="18" width="10.44140625" style="23" customWidth="1"/>
+    <col min="19" max="19" width="12.5546875" style="23" customWidth="1"/>
+    <col min="20" max="20" width="10.6640625" style="32"/>
+    <col min="21" max="21" width="10.6640625" style="31"/>
+    <col min="22" max="22" width="10.6640625" style="32"/>
+    <col min="23" max="23" width="14.6640625" style="22" customWidth="1"/>
+    <col min="24" max="24" width="13.77734375" style="22" customWidth="1"/>
+    <col min="25" max="26" width="10.6640625" style="22"/>
+    <col min="27" max="27" width="22.109375" style="22" customWidth="1"/>
+    <col min="28" max="28" width="24.5546875" style="22" customWidth="1"/>
+    <col min="29" max="29" width="20.5546875" style="22" customWidth="1"/>
+    <col min="30" max="30" width="14.109375" style="27" customWidth="1"/>
+    <col min="31" max="32" width="40.77734375" style="34" customWidth="1"/>
+    <col min="33" max="16384" width="10.6640625" style="35"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:58" customFormat="1" x14ac:dyDescent="0.3">
@@ -1185,21 +1030,21 @@
       <c r="BF1" s="3"/>
     </row>
     <row r="2" spans="1:58" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
-      <c r="K2" s="42"/>
-      <c r="L2" s="42"/>
-      <c r="M2" s="42"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="36"/>
+      <c r="L2" s="36"/>
+      <c r="M2" s="36"/>
       <c r="N2" s="2"/>
       <c r="O2" s="4"/>
       <c r="P2" s="3"/>
@@ -1247,21 +1092,21 @@
       <c r="BF2" s="3"/>
     </row>
     <row r="3" spans="1:58" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="43"/>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="43"/>
-      <c r="I3" s="43"/>
-      <c r="J3" s="43"/>
-      <c r="K3" s="43"/>
-      <c r="L3" s="43"/>
-      <c r="M3" s="43"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="37"/>
+      <c r="H3" s="37"/>
+      <c r="I3" s="37"/>
+      <c r="J3" s="37"/>
+      <c r="K3" s="37"/>
+      <c r="L3" s="37"/>
+      <c r="M3" s="37"/>
       <c r="N3" s="1"/>
       <c r="O3" s="5"/>
       <c r="P3" s="3"/>
@@ -1309,19 +1154,19 @@
       <c r="BF3" s="3"/>
     </row>
     <row r="4" spans="1:58" customFormat="1" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="42"/>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="42"/>
-      <c r="I4" s="42"/>
-      <c r="J4" s="42"/>
-      <c r="K4" s="42"/>
-      <c r="L4" s="42"/>
-      <c r="M4" s="42"/>
+      <c r="A4" s="36"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
+      <c r="M4" s="36"/>
       <c r="N4" s="4"/>
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
@@ -1388,7 +1233,7 @@
     <row r="6" spans="1:58" customFormat="1" ht="18" x14ac:dyDescent="0.3">
       <c r="A6" s="6"/>
       <c r="B6" s="6"/>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="29" t="s">
         <v>2</v>
       </c>
       <c r="D6" s="9"/>
@@ -1398,7 +1243,7 @@
       <c r="H6" s="10"/>
       <c r="I6" s="6"/>
       <c r="J6" s="6"/>
-      <c r="K6" s="33" t="s">
+      <c r="K6" s="28" t="s">
         <v>3</v>
       </c>
       <c r="L6" s="11"/>
@@ -1421,119 +1266,119 @@
       <c r="T7" s="21"/>
     </row>
     <row r="8" spans="1:58" s="18" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="36" t="s">
+      <c r="B8" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="36" t="s">
+      <c r="C8" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="36" t="s">
+      <c r="D8" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="36" t="s">
+      <c r="E8" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="36" t="s">
+      <c r="F8" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="G8" s="44" t="s">
+      <c r="G8" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="44"/>
-      <c r="I8" s="36" t="s">
+      <c r="H8" s="39"/>
+      <c r="I8" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="J8" s="36" t="s">
+      <c r="J8" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="K8" s="36" t="s">
+      <c r="K8" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="L8" s="36" t="s">
+      <c r="L8" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="M8" s="36" t="s">
+      <c r="M8" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="N8" s="36" t="s">
+      <c r="N8" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="O8" s="36" t="s">
+      <c r="O8" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="P8" s="36" t="s">
+      <c r="P8" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="Q8" s="38"/>
-      <c r="R8" s="36" t="s">
+      <c r="Q8" s="41"/>
+      <c r="R8" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="S8" s="36"/>
-      <c r="T8" s="36" t="s">
+      <c r="S8" s="38"/>
+      <c r="T8" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="U8" s="36" t="s">
+      <c r="U8" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="V8" s="36" t="s">
+      <c r="V8" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="W8" s="37" t="s">
+      <c r="W8" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="X8" s="39" t="s">
+      <c r="X8" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="Y8" s="40" t="s">
+      <c r="Y8" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="Z8" s="37" t="s">
+      <c r="Z8" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="AA8" s="37" t="s">
+      <c r="AA8" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="AB8" s="37" t="s">
+      <c r="AB8" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="AC8" s="37" t="s">
+      <c r="AC8" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="AD8" s="36" t="s">
+      <c r="AD8" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="AE8" s="35" t="s">
+      <c r="AE8" s="43" t="s">
         <v>35</v>
       </c>
-      <c r="AF8" s="35"/>
+      <c r="AF8" s="43"/>
     </row>
     <row r="9" spans="1:58" s="18" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="36"/>
-      <c r="B9" s="36"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
+      <c r="A9" s="38"/>
+      <c r="B9" s="38"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="38"/>
+      <c r="F9" s="38"/>
       <c r="G9" s="20" t="s">
         <v>13</v>
       </c>
       <c r="H9" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="36"/>
-      <c r="J9" s="36"/>
-      <c r="K9" s="36"/>
-      <c r="L9" s="36"/>
-      <c r="M9" s="36"/>
-      <c r="N9" s="36"/>
-      <c r="O9" s="36"/>
+      <c r="I9" s="38"/>
+      <c r="J9" s="38"/>
+      <c r="K9" s="38"/>
+      <c r="L9" s="38"/>
+      <c r="M9" s="38"/>
+      <c r="N9" s="38"/>
+      <c r="O9" s="38"/>
       <c r="P9" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="Q9" s="29" t="s">
+      <c r="Q9" s="26" t="s">
         <v>23</v>
       </c>
       <c r="R9" s="19" t="s">
@@ -1542,31 +1387,50 @@
       <c r="S9" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="T9" s="36"/>
-      <c r="U9" s="36"/>
-      <c r="V9" s="41"/>
-      <c r="W9" s="37"/>
-      <c r="X9" s="39"/>
-      <c r="Y9" s="40"/>
-      <c r="Z9" s="37"/>
-      <c r="AA9" s="37"/>
-      <c r="AB9" s="37"/>
-      <c r="AC9" s="37"/>
-      <c r="AD9" s="36"/>
-      <c r="AE9" s="19" t="s">
+      <c r="T9" s="38"/>
+      <c r="U9" s="38"/>
+      <c r="V9" s="38"/>
+      <c r="W9" s="40"/>
+      <c r="X9" s="40"/>
+      <c r="Y9" s="42"/>
+      <c r="Z9" s="42"/>
+      <c r="AA9" s="40"/>
+      <c r="AB9" s="40"/>
+      <c r="AC9" s="40"/>
+      <c r="AD9" s="38"/>
+      <c r="AE9" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="AF9" s="19" t="s">
+      <c r="AF9" s="30" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:58" x14ac:dyDescent="0.2">
-      <c r="J12" s="23" t="s">
+      <c r="J12" s="33" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="AE8:AF8"/>
+    <mergeCell ref="AD8:AD9"/>
+    <mergeCell ref="Z8:Z9"/>
+    <mergeCell ref="AA8:AA9"/>
+    <mergeCell ref="AB8:AB9"/>
+    <mergeCell ref="AC8:AC9"/>
+    <mergeCell ref="W8:W9"/>
+    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="R8:S8"/>
+    <mergeCell ref="X8:X9"/>
+    <mergeCell ref="Y8:Y9"/>
+    <mergeCell ref="T8:T9"/>
+    <mergeCell ref="U8:U9"/>
+    <mergeCell ref="V8:V9"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="K8:K9"/>
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A3:M3"/>
     <mergeCell ref="J8:J9"/>
@@ -1579,56 +1443,52 @@
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="A4:M4"/>
-    <mergeCell ref="O8:O9"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="W8:W9"/>
-    <mergeCell ref="P8:Q8"/>
-    <mergeCell ref="R8:S8"/>
-    <mergeCell ref="X8:X9"/>
-    <mergeCell ref="Y8:Y9"/>
-    <mergeCell ref="T8:T9"/>
-    <mergeCell ref="U8:U9"/>
-    <mergeCell ref="V8:V9"/>
-    <mergeCell ref="AE8:AF8"/>
-    <mergeCell ref="AD8:AD9"/>
-    <mergeCell ref="Z8:Z9"/>
-    <mergeCell ref="AA8:AA9"/>
-    <mergeCell ref="AB8:AB9"/>
-    <mergeCell ref="AC8:AC9"/>
   </mergeCells>
+  <conditionalFormatting sqref="A10:AF1048576">
+    <cfRule type="expression" dxfId="9" priority="3">
+      <formula>$AA10="ANULADO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G10:H1048576">
+    <cfRule type="expression" dxfId="8" priority="2">
+      <formula>$A10&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="T10:T1048576">
-    <cfRule type="cellIs" dxfId="13" priority="7" stopIfTrue="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="10" stopIfTrue="1" operator="greaterThan">
       <formula>0.01</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T2186:T1048576">
-    <cfRule type="expression" dxfId="12" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="9" stopIfTrue="1">
       <formula>$AD2186="-"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U10 U11:V1048576">
-    <cfRule type="expression" dxfId="11" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="8" stopIfTrue="1">
       <formula>$AD10="-"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="U10:V1048576">
+    <cfRule type="expression" dxfId="4" priority="1">
+      <formula>$A10&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="V10:V1048576">
-    <cfRule type="expression" dxfId="10" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="7" stopIfTrue="1">
       <formula>$AD10="-"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA10:AA1048576">
-    <cfRule type="expression" dxfId="9" priority="1">
+    <cfRule type="expression" dxfId="2" priority="4">
       <formula>"ANULADO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD10:AD1048576">
-    <cfRule type="containsText" dxfId="8" priority="2" operator="containsText" text="RUMA">
+    <cfRule type="containsText" dxfId="1" priority="5" operator="containsText" text="RUMA">
       <formula>NOT(ISERROR(SEARCH("RUMA",AD10)))</formula>
     </cfRule>
-    <cfRule type="top10" dxfId="7" priority="3" rank="1000"/>
+    <cfRule type="top10" dxfId="0" priority="6" rank="1000"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: actualizar plantilla chancado
</commit_message>
<xml_diff>
--- a/chancado/analytica/Report/Lote-Export-Base.xlsx
+++ b/chancado/analytica/Report/Lote-Export-Base.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\projects\minersoft-projects\minersoft\acopio-chancado-api\Acopio.Chancado.Apis\Report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\projects\minersoft-projects\minersoft\acopio-project-configuration\chancado\analytica\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7AE4F18-A650-4594-B271-F045A1860F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7B34D37-BB82-431C-9C0E-EA27BC41E335}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28908" yWindow="-108" windowWidth="29016" windowHeight="15696" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -291,7 +291,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -313,12 +313,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -475,17 +469,13 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="16" fontId="17" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="24" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -505,29 +495,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="16" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="22" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="22" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="25">
@@ -557,7 +551,7 @@
     <cellStyle name="Normal 2 2 2 2" xfId="24" xr:uid="{7D02EEDF-F966-42E2-BF75-AE97ED01237A}"/>
     <cellStyle name="Normal 3" xfId="23" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="33">
     <dxf>
       <font>
         <b/>
@@ -593,9 +587,266 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FFCCFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF0000FF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor auto="1"/>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="1"/>
+        </left>
+        <right style="thin">
+          <color theme="1"/>
+        </right>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom style="thin">
+          <color theme="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF5D5D"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF0000FF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor auto="1"/>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <numFmt numFmtId="21" formatCode="dd\-mmm"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FF00FF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color theme="1"/>
+        </left>
+        <right style="thin">
+          <color theme="1"/>
+        </right>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom style="thin">
+          <color theme="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF5D5D"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <numFmt numFmtId="21" formatCode="dd\-mmm"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FF00FF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF0000FF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor auto="1"/>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -740,6 +991,7 @@
       <rgbColor rgb="00333333"/>
     </indexedColors>
     <mruColors>
+      <color rgb="FF0000FF"/>
       <color rgb="FFFF5D5D"/>
       <color rgb="FF00FF00"/>
       <color rgb="FFC0C0C0"/>
@@ -939,34 +1191,34 @@
     <col min="1" max="1" width="6.77734375" style="22" customWidth="1"/>
     <col min="2" max="2" width="19.77734375" style="23" customWidth="1"/>
     <col min="3" max="3" width="19.5546875" style="24" customWidth="1"/>
-    <col min="4" max="4" width="19.5546875" style="33" customWidth="1"/>
-    <col min="5" max="5" width="16.6640625" style="33" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.77734375" style="33" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.5546875" style="32" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" style="32" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.77734375" style="32" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.5546875" style="22" customWidth="1"/>
     <col min="8" max="8" width="10" style="22" customWidth="1"/>
-    <col min="9" max="9" width="9.109375" style="33" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="44.88671875" style="33" customWidth="1"/>
-    <col min="11" max="11" width="25.77734375" style="33" customWidth="1"/>
-    <col min="12" max="12" width="52.5546875" style="33" customWidth="1"/>
-    <col min="13" max="13" width="19.88671875" style="33" customWidth="1"/>
-    <col min="14" max="14" width="15" style="33" customWidth="1"/>
-    <col min="15" max="15" width="17.33203125" style="33" customWidth="1"/>
+    <col min="9" max="9" width="9.109375" style="32" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="44.88671875" style="32" customWidth="1"/>
+    <col min="11" max="11" width="25.77734375" style="32" customWidth="1"/>
+    <col min="12" max="12" width="52.5546875" style="32" customWidth="1"/>
+    <col min="13" max="13" width="19.88671875" style="32" customWidth="1"/>
+    <col min="14" max="14" width="15" style="32" customWidth="1"/>
+    <col min="15" max="15" width="17.33203125" style="32" customWidth="1"/>
     <col min="16" max="16" width="10.33203125" style="25" customWidth="1"/>
     <col min="17" max="17" width="12.21875" style="25" customWidth="1"/>
     <col min="18" max="18" width="10.44140625" style="23" customWidth="1"/>
     <col min="19" max="19" width="12.5546875" style="23" customWidth="1"/>
-    <col min="20" max="20" width="10.6640625" style="32"/>
-    <col min="21" max="21" width="10.6640625" style="31"/>
-    <col min="22" max="22" width="10.6640625" style="32"/>
+    <col min="20" max="20" width="10.6640625" style="31"/>
+    <col min="21" max="21" width="10.6640625" style="30"/>
+    <col min="22" max="22" width="10.6640625" style="31"/>
     <col min="23" max="23" width="14.6640625" style="22" customWidth="1"/>
     <col min="24" max="24" width="13.77734375" style="22" customWidth="1"/>
     <col min="25" max="26" width="10.6640625" style="22"/>
     <col min="27" max="27" width="22.109375" style="22" customWidth="1"/>
     <col min="28" max="28" width="24.5546875" style="22" customWidth="1"/>
     <col min="29" max="29" width="20.5546875" style="22" customWidth="1"/>
-    <col min="30" max="30" width="14.109375" style="27" customWidth="1"/>
-    <col min="31" max="32" width="40.77734375" style="34" customWidth="1"/>
-    <col min="33" max="16384" width="10.6640625" style="35"/>
+    <col min="30" max="30" width="14.109375" style="35" customWidth="1"/>
+    <col min="31" max="32" width="40.77734375" style="33" customWidth="1"/>
+    <col min="33" max="16384" width="10.6640625" style="34"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:58" customFormat="1" x14ac:dyDescent="0.3">
@@ -1030,21 +1282,21 @@
       <c r="BF1" s="3"/>
     </row>
     <row r="2" spans="1:58" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="41"/>
+      <c r="L2" s="41"/>
+      <c r="M2" s="41"/>
       <c r="N2" s="2"/>
       <c r="O2" s="4"/>
       <c r="P2" s="3"/>
@@ -1092,21 +1344,21 @@
       <c r="BF2" s="3"/>
     </row>
     <row r="3" spans="1:58" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="37" t="s">
+      <c r="A3" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="37"/>
-      <c r="H3" s="37"/>
-      <c r="I3" s="37"/>
-      <c r="J3" s="37"/>
-      <c r="K3" s="37"/>
-      <c r="L3" s="37"/>
-      <c r="M3" s="37"/>
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
+      <c r="H3" s="42"/>
+      <c r="I3" s="42"/>
+      <c r="J3" s="42"/>
+      <c r="K3" s="42"/>
+      <c r="L3" s="42"/>
+      <c r="M3" s="42"/>
       <c r="N3" s="1"/>
       <c r="O3" s="5"/>
       <c r="P3" s="3"/>
@@ -1154,19 +1406,19 @@
       <c r="BF3" s="3"/>
     </row>
     <row r="4" spans="1:58" customFormat="1" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="36"/>
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="36"/>
-      <c r="L4" s="36"/>
-      <c r="M4" s="36"/>
+      <c r="A4" s="41"/>
+      <c r="B4" s="41"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="41"/>
+      <c r="K4" s="41"/>
+      <c r="L4" s="41"/>
+      <c r="M4" s="41"/>
       <c r="N4" s="4"/>
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
@@ -1233,7 +1485,7 @@
     <row r="6" spans="1:58" customFormat="1" ht="18" x14ac:dyDescent="0.3">
       <c r="A6" s="6"/>
       <c r="B6" s="6"/>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="28" t="s">
         <v>2</v>
       </c>
       <c r="D6" s="9"/>
@@ -1243,7 +1495,7 @@
       <c r="H6" s="10"/>
       <c r="I6" s="6"/>
       <c r="J6" s="6"/>
-      <c r="K6" s="28" t="s">
+      <c r="K6" s="27" t="s">
         <v>3</v>
       </c>
       <c r="L6" s="11"/>
@@ -1266,115 +1518,115 @@
       <c r="T7" s="21"/>
     </row>
     <row r="8" spans="1:58" s="18" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="38" t="s">
+      <c r="B8" s="37" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="38" t="s">
+      <c r="C8" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="38" t="s">
+      <c r="D8" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="38" t="s">
+      <c r="E8" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="38" t="s">
+      <c r="F8" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="G8" s="39" t="s">
+      <c r="G8" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="39"/>
-      <c r="I8" s="38" t="s">
+      <c r="H8" s="43"/>
+      <c r="I8" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="J8" s="38" t="s">
+      <c r="J8" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="K8" s="38" t="s">
+      <c r="K8" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="L8" s="38" t="s">
+      <c r="L8" s="37" t="s">
         <v>18</v>
       </c>
-      <c r="M8" s="38" t="s">
+      <c r="M8" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="N8" s="38" t="s">
+      <c r="N8" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="O8" s="38" t="s">
+      <c r="O8" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="P8" s="38" t="s">
+      <c r="P8" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="Q8" s="41"/>
-      <c r="R8" s="38" t="s">
+      <c r="Q8" s="40"/>
+      <c r="R8" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="S8" s="38"/>
-      <c r="T8" s="38" t="s">
+      <c r="S8" s="37"/>
+      <c r="T8" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="U8" s="38" t="s">
+      <c r="U8" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="V8" s="38" t="s">
+      <c r="V8" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="W8" s="40" t="s">
+      <c r="W8" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="X8" s="40" t="s">
+      <c r="X8" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="Y8" s="42" t="s">
+      <c r="Y8" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="Z8" s="42" t="s">
+      <c r="Z8" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="AA8" s="40" t="s">
+      <c r="AA8" s="39" t="s">
         <v>32</v>
       </c>
-      <c r="AB8" s="40" t="s">
+      <c r="AB8" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="AC8" s="40" t="s">
+      <c r="AC8" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="AD8" s="38" t="s">
+      <c r="AD8" s="37" t="s">
         <v>37</v>
       </c>
-      <c r="AE8" s="43" t="s">
+      <c r="AE8" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="AF8" s="43"/>
+      <c r="AF8" s="36"/>
     </row>
     <row r="9" spans="1:58" s="18" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="38"/>
-      <c r="B9" s="38"/>
-      <c r="C9" s="38"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="38"/>
-      <c r="F9" s="38"/>
+      <c r="A9" s="37"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
       <c r="G9" s="20" t="s">
         <v>13</v>
       </c>
       <c r="H9" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="38"/>
-      <c r="J9" s="38"/>
-      <c r="K9" s="38"/>
-      <c r="L9" s="38"/>
-      <c r="M9" s="38"/>
-      <c r="N9" s="38"/>
-      <c r="O9" s="38"/>
+      <c r="I9" s="37"/>
+      <c r="J9" s="37"/>
+      <c r="K9" s="37"/>
+      <c r="L9" s="37"/>
+      <c r="M9" s="37"/>
+      <c r="N9" s="37"/>
+      <c r="O9" s="37"/>
       <c r="P9" s="19" t="s">
         <v>22</v>
       </c>
@@ -1387,50 +1639,31 @@
       <c r="S9" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="T9" s="38"/>
-      <c r="U9" s="38"/>
-      <c r="V9" s="38"/>
-      <c r="W9" s="40"/>
-      <c r="X9" s="40"/>
-      <c r="Y9" s="42"/>
-      <c r="Z9" s="42"/>
-      <c r="AA9" s="40"/>
-      <c r="AB9" s="40"/>
-      <c r="AC9" s="40"/>
-      <c r="AD9" s="38"/>
-      <c r="AE9" s="30" t="s">
+      <c r="T9" s="37"/>
+      <c r="U9" s="37"/>
+      <c r="V9" s="37"/>
+      <c r="W9" s="39"/>
+      <c r="X9" s="39"/>
+      <c r="Y9" s="38"/>
+      <c r="Z9" s="38"/>
+      <c r="AA9" s="39"/>
+      <c r="AB9" s="39"/>
+      <c r="AC9" s="39"/>
+      <c r="AD9" s="37"/>
+      <c r="AE9" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="AF9" s="30" t="s">
+      <c r="AF9" s="29" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:58" x14ac:dyDescent="0.2">
-      <c r="J12" s="33" t="s">
+      <c r="J12" s="32" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="AE8:AF8"/>
-    <mergeCell ref="AD8:AD9"/>
-    <mergeCell ref="Z8:Z9"/>
-    <mergeCell ref="AA8:AA9"/>
-    <mergeCell ref="AB8:AB9"/>
-    <mergeCell ref="AC8:AC9"/>
-    <mergeCell ref="W8:W9"/>
-    <mergeCell ref="P8:Q8"/>
-    <mergeCell ref="R8:S8"/>
-    <mergeCell ref="X8:X9"/>
-    <mergeCell ref="Y8:Y9"/>
-    <mergeCell ref="T8:T9"/>
-    <mergeCell ref="U8:U9"/>
-    <mergeCell ref="V8:V9"/>
-    <mergeCell ref="O8:O9"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="K8:K9"/>
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A3:M3"/>
     <mergeCell ref="J8:J9"/>
@@ -1443,52 +1676,74 @@
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="A4:M4"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="W8:W9"/>
+    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="R8:S8"/>
+    <mergeCell ref="X8:X9"/>
+    <mergeCell ref="Y8:Y9"/>
+    <mergeCell ref="T8:T9"/>
+    <mergeCell ref="U8:U9"/>
+    <mergeCell ref="V8:V9"/>
+    <mergeCell ref="AE8:AF8"/>
+    <mergeCell ref="AD8:AD9"/>
+    <mergeCell ref="Z8:Z9"/>
+    <mergeCell ref="AA8:AA9"/>
+    <mergeCell ref="AB8:AB9"/>
+    <mergeCell ref="AC8:AC9"/>
   </mergeCells>
   <conditionalFormatting sqref="A10:AF1048576">
-    <cfRule type="expression" dxfId="9" priority="3">
+    <cfRule type="expression" dxfId="21" priority="1">
       <formula>$AA10="ANULADO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G10:H1048576">
-    <cfRule type="expression" dxfId="8" priority="2">
+    <cfRule type="expression" dxfId="20" priority="3">
       <formula>$A10&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T10:T1048576">
-    <cfRule type="cellIs" dxfId="7" priority="10" stopIfTrue="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="19" priority="11" stopIfTrue="1" operator="greaterThan">
       <formula>0.01</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T2186:T1048576">
-    <cfRule type="expression" dxfId="6" priority="9" stopIfTrue="1">
+    <cfRule type="expression" dxfId="18" priority="10" stopIfTrue="1">
       <formula>$AD2186="-"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U10 U11:V1048576">
-    <cfRule type="expression" dxfId="5" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="17" priority="9" stopIfTrue="1">
       <formula>$AD10="-"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U10:V1048576">
-    <cfRule type="expression" dxfId="4" priority="1">
+  <conditionalFormatting sqref="V10:V1048576">
+    <cfRule type="expression" dxfId="16" priority="8" stopIfTrue="1">
+      <formula>$AD10="-"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="11" priority="4">
       <formula>$A10&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V10:V1048576">
-    <cfRule type="expression" dxfId="3" priority="7" stopIfTrue="1">
-      <formula>$AD10="-"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="AA10:AA1048576">
-    <cfRule type="expression" dxfId="2" priority="4">
+    <cfRule type="expression" dxfId="15" priority="5">
       <formula>"ANULADO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD10:AD1048576">
-    <cfRule type="containsText" dxfId="1" priority="5" operator="containsText" text="RUMA">
+    <cfRule type="containsText" dxfId="14" priority="6" operator="containsText" text="RUMA">
       <formula>NOT(ISERROR(SEARCH("RUMA",AD10)))</formula>
     </cfRule>
-    <cfRule type="top10" dxfId="0" priority="6" rank="1000"/>
+    <cfRule type="top10" dxfId="13" priority="7" rank="1000"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U10:U1048576">
+    <cfRule type="expression" dxfId="12" priority="2">
+      <formula>$A10&lt;&gt;""</formula>
+    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>